<commit_message>
Update contact email to justin@goldentide.cloud and add Outlook signature
Refresh site Contact details and all downloadable flyers, cards,
invoices, and quotes; add Outlook HTML signature for clients/mail.
</commit_message>
<xml_diff>
--- a/public/downloads/invoice-template.xlsx
+++ b/public/downloads/invoice-template.xlsx
@@ -707,7 +707,7 @@
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>+685 770 3733  ·  justinvs@live.co.za</t>
+          <t>+685 770 3733  ·  justin@goldentide.cloud</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -1012,7 +1012,7 @@
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>Payment due within 14 days of invoice date unless otherwise agreed. Thank you for your business. For questions about this invoice, contact Justin at +685 770 3733 or justinvs@live.co.za.</t>
+          <t>Payment due within 14 days of invoice date unless otherwise agreed. Thank you for your business. For questions about this invoice, contact Justin at +685 770 3733 or justin@goldentide.cloud.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync marketing downloads with official logo branding
Refresh flyer, business card, invoice, and quote PDFs/DOCX plus the
logo asset served from /downloads.
</commit_message>
<xml_diff>
--- a/public/downloads/invoice-template.xlsx
+++ b/public/downloads/invoice-template.xlsx
@@ -150,7 +150,7 @@
   <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="8"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -265,6 +265,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="514350" cy="514350"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -568,7 +598,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GOLDEN TIDE</t>
@@ -581,7 +611,7 @@
       <c r="F1" s="2" t="n"/>
       <c r="G1" s="2" t="n"/>
     </row>
-    <row r="2" ht="10" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
@@ -1047,5 +1077,6 @@
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>